<commit_message>
First look of MVP April 2nd with preset of users and passwords and stores data from excels and dynamic daily active visitors
</commit_message>
<xml_diff>
--- a/data/daily_visitor_status_sample_10.xlsx
+++ b/data/daily_visitor_status_sample_10.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="daily_status" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -27,23 +27,17 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -51,14 +45,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -134,51 +134,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>OpenAI</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>Format: YYYY-MM-DD</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>Must match an existing visitor profile.</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>Actual capacity for that day.</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>TRUE/FALSE</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DailyVisitorStatus10Template" displayName="DailyVisitorStatus10Template" ref="A1:F11" headerRowCount="1">
-  <autoFilter ref="A1:F11"/>
-  <tableColumns count="6">
-    <tableColumn id="1" name="work_date"/>
-    <tableColumn id="2" name="visitor_code"/>
-    <tableColumn id="3" name="start_lat"/>
-    <tableColumn id="4" name="start_lon"/>
-    <tableColumn id="5" name="capacity"/>
-    <tableColumn id="6" name="is_active_today"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -470,16 +425,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -489,25 +436,35 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>username</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>visitor_code</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>full_name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>start_lat</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>start_lon</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>capacity</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>is_active_today</t>
         </is>
@@ -516,248 +473,344 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>visitor1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>VIS-001</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>35.777114</v>
-      </c>
-      <c r="D2" t="n">
-        <v>51.399439</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ویزیتور 01</t>
+        </is>
       </c>
       <c r="E2" t="n">
-        <v>30</v>
-      </c>
-      <c r="F2" t="b">
+        <v>35.67</v>
+      </c>
+      <c r="F2" t="n">
+        <v>51.33</v>
+      </c>
+      <c r="G2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>visitor2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>VIS-002</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>35.745218</v>
-      </c>
-      <c r="D3" t="n">
-        <v>51.365308</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ویزیتور 02</t>
+        </is>
       </c>
       <c r="E3" t="n">
-        <v>30</v>
-      </c>
-      <c r="F3" t="b">
+        <v>35.68</v>
+      </c>
+      <c r="F3" t="n">
+        <v>51.34</v>
+      </c>
+      <c r="G3" t="n">
+        <v>30</v>
+      </c>
+      <c r="H3" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>visitor3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>VIS-003</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>35.711991</v>
-      </c>
-      <c r="D4" t="n">
-        <v>51.546789</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ویزیتور 03</t>
+        </is>
       </c>
       <c r="E4" t="n">
-        <v>30</v>
-      </c>
-      <c r="F4" t="b">
+        <v>35.69</v>
+      </c>
+      <c r="F4" t="n">
+        <v>51.35</v>
+      </c>
+      <c r="G4" t="n">
+        <v>30</v>
+      </c>
+      <c r="H4" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>visitor4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>VIS-004</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>35.743584</v>
-      </c>
-      <c r="D5" t="n">
-        <v>51.241966</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ویزیتور 04</t>
+        </is>
       </c>
       <c r="E5" t="n">
-        <v>30</v>
-      </c>
-      <c r="F5" t="b">
+        <v>35.7</v>
+      </c>
+      <c r="F5" t="n">
+        <v>51.36</v>
+      </c>
+      <c r="G5" t="n">
+        <v>30</v>
+      </c>
+      <c r="H5" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>visitor5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>VIS-005</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>35.660157</v>
-      </c>
-      <c r="D6" t="n">
-        <v>51.39285</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ویزیتور 05</t>
+        </is>
       </c>
       <c r="E6" t="n">
-        <v>30</v>
-      </c>
-      <c r="F6" t="b">
+        <v>35.71</v>
+      </c>
+      <c r="F6" t="n">
+        <v>51.37</v>
+      </c>
+      <c r="G6" t="n">
+        <v>30</v>
+      </c>
+      <c r="H6" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>visitor6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>VIS-006</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>35.780839</v>
-      </c>
-      <c r="D7" t="n">
-        <v>51.431808</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ویزیتور 06</t>
+        </is>
       </c>
       <c r="E7" t="n">
-        <v>30</v>
-      </c>
-      <c r="F7" t="b">
+        <v>35.72</v>
+      </c>
+      <c r="F7" t="n">
+        <v>51.38</v>
+      </c>
+      <c r="G7" t="n">
+        <v>30</v>
+      </c>
+      <c r="H7" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>visitor7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>VIS-007</t>
         </is>
       </c>
-      <c r="C8" t="n">
-        <v>35.715959</v>
-      </c>
-      <c r="D8" t="n">
-        <v>51.330832</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ویزیتور 07</t>
+        </is>
       </c>
       <c r="E8" t="n">
-        <v>30</v>
-      </c>
-      <c r="F8" t="b">
+        <v>35.73</v>
+      </c>
+      <c r="F8" t="n">
+        <v>51.39</v>
+      </c>
+      <c r="G8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>visitor8</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>VIS-008</t>
         </is>
       </c>
-      <c r="C9" t="n">
-        <v>35.741207</v>
-      </c>
-      <c r="D9" t="n">
-        <v>51.465581</v>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ویزیتور 08</t>
+        </is>
       </c>
       <c r="E9" t="n">
-        <v>30</v>
-      </c>
-      <c r="F9" t="b">
+        <v>35.74</v>
+      </c>
+      <c r="F9" t="n">
+        <v>51.4</v>
+      </c>
+      <c r="G9" t="n">
+        <v>30</v>
+      </c>
+      <c r="H9" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>visitor9</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>VIS-009</t>
         </is>
       </c>
-      <c r="C10" t="n">
-        <v>35.719552</v>
-      </c>
-      <c r="D10" t="n">
-        <v>51.27121</v>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ویزیتور 09</t>
+        </is>
       </c>
       <c r="E10" t="n">
-        <v>30</v>
-      </c>
-      <c r="F10" t="b">
+        <v>35.75</v>
+      </c>
+      <c r="F10" t="n">
+        <v>51.41</v>
+      </c>
+      <c r="G10" t="n">
+        <v>30</v>
+      </c>
+      <c r="H10" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>visitor10</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>VIS-010</t>
         </is>
       </c>
-      <c r="C11" t="n">
-        <v>35.654035</v>
-      </c>
-      <c r="D11" t="n">
-        <v>51.360367</v>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ویزیتور 10</t>
+        </is>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" t="b">
-        <v>0</v>
+        <v>35.76</v>
+      </c>
+      <c r="F11" t="n">
+        <v>51.42</v>
+      </c>
+      <c r="G11" t="n">
+        <v>30</v>
+      </c>
+      <c r="H11" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>